<commit_message>
zadnji popravki + rezultati
</commit_message>
<xml_diff>
--- a/Rezultati/Časi.xlsx
+++ b/Rezultati/Časi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zavse\Desktop\studij\3.letnik\DiplomskaNaloga\Faza1\Rezultati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573CB4FE-513D-4197-9E95-A2A48A07A576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80545043-7148-4F3D-B8FB-9FE381201FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20496" yWindow="2520" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20256" yWindow="2916" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="časi" sheetId="1" r:id="rId1"/>
@@ -421,7 +421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -437,7 +437,7 @@
     <col min="12" max="12" width="6.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +472,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -507,8 +507,12 @@
         <f>SUM(C2,E2,G2,I2)</f>
         <v>0.48333333333333334</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M2">
+        <f>SUM(D2,F2,H2,J2)</f>
+        <v>1777</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -533,12 +537,22 @@
       <c r="H3">
         <v>286</v>
       </c>
+      <c r="I3" s="1">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="J3">
+        <v>35</v>
+      </c>
       <c r="L3" s="1">
-        <f t="shared" ref="L3:L11" si="0">SUM(C3,E3,G3)</f>
+        <f t="shared" ref="L3:L10" si="0">SUM(C3,E3,G3)</f>
         <v>0.32361111111111113</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3">
+        <f t="shared" ref="M3:M9" si="1">SUM(D3,F3,H3,J3)</f>
+        <v>933</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -563,12 +577,17 @@
       <c r="H4">
         <v>425</v>
       </c>
+      <c r="I4" s="1"/>
       <c r="L4" s="1">
         <f t="shared" si="0"/>
         <v>0.41041666666666665</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4">
+        <f t="shared" si="1"/>
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -597,8 +616,12 @@
         <f t="shared" si="0"/>
         <v>0.24444444444444444</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5">
+        <f t="shared" si="1"/>
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -622,13 +645,23 @@
       </c>
       <c r="H6">
         <v>327</v>
+      </c>
+      <c r="I6" s="1">
+        <v>8.4027777777777785E-2</v>
+      </c>
+      <c r="J6">
+        <v>34</v>
       </c>
       <c r="L6" s="1">
         <f t="shared" si="0"/>
         <v>0.28541666666666665</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6">
+        <f t="shared" si="1"/>
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -652,13 +685,23 @@
       </c>
       <c r="H7">
         <v>407</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.11388888888888889</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" si="0"/>
         <v>0.32430555555555557</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M7">
+        <f t="shared" si="1"/>
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -687,8 +730,12 @@
         <f t="shared" si="0"/>
         <v>0.28194444444444444</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M8">
+        <f t="shared" si="1"/>
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -712,13 +759,23 @@
       </c>
       <c r="H9">
         <v>271</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0.11388888888888889</v>
+      </c>
+      <c r="J9">
+        <v>34</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="0"/>
         <v>0.29166666666666669</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M9">
+        <f t="shared" si="1"/>
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -742,13 +799,23 @@
       </c>
       <c r="H10">
         <v>433</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.12430555555555556</v>
+      </c>
+      <c r="J10">
+        <v>7</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="0"/>
         <v>0.39374999999999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M10">
+        <f>SUM(D10,F10,H10,J10)</f>
+        <v>1414</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="L11" s="1"/>
     </row>
   </sheetData>
@@ -852,11 +919,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D8:E8"/>
@@ -865,6 +927,11 @@
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>